<commit_message>
feat(config): map Polity topic thread ID to 3
- Update config.xlsx with Topic_Thread_ID = 3 for Polity subject
- Tested Telegram bot communication and poll delivery to forum topic
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -402,7 +402,7 @@
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="22.83203125" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
   </cols>
@@ -434,8 +434,8 @@
       <c r="B2" t="str">
         <v>⚖️</v>
       </c>
-      <c r="C2" t="str">
-        <v/>
+      <c r="C2">
+        <v>3</v>
       </c>
       <c r="D2" t="str">
         <v>0 */2 * * *</v>

</xml_diff>

<commit_message>
feat(economy): map topic ID 8, support long poll questions, and post AP-Green question
- Map Topic_Thread_ID = 8 for Economy in config.xlsx (https://t.me/c/3814998988/8)
- Enhance src/telegram.js to support long questions (>290 chars) by posting the full statement prompt as an HTML topic message followed by the quiz poll
- Add escapeHtml utility to prevent HTML entity parsing errors in Telegram messages
- Fix row index tracking in src/excel.js, send.js, and schedule.js to ensure accurate 0-based and 1-based row synchronization
- Add AP-Green forest cover question to questions.xlsx under Economy sheet
- Post AP-Green quiz question to Economy forum topic (Thread ID: 8) and mark as posted
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -454,8 +454,8 @@
       <c r="B3" t="str">
         <v>💰</v>
       </c>
-      <c r="C3" t="str">
-        <v/>
+      <c r="C3">
+        <v>8</v>
       </c>
       <c r="D3" t="str">
         <v>0 */3 * * *</v>

</xml_diff>

<commit_message>
feat(topics): save created Telegram topic thread IDs for all 16 APPSC subjects
- Executed setup.js against supergroup 'Sadhana APPSC' (-1004476950050)
- Successfully created 16 forum topics on the Telegram supergroup sidebar:
  * 📜 History (Thread ID: 6)
  * 🏛️ AP History (Thread ID: 7)
  * 🌍 Geography (Thread ID: 8)
  * 🗺️ AP Geography (Thread ID: 9)
  * 💰 Economy (Thread ID: 10)
  * 📈 AP Economy (Thread ID: 11)
  * ⚖️ Polity (Thread ID: 12)
  * 👥 Society (Thread ID: 13)
  * 📰 Current Affairs (Thread ID: 14)
  * 🚀 Science and Technology (Thread ID: 15)
  * 🧬 Biology (Thread ID: 16)
  * 🧪 Chemistry (Thread ID: 17)
  * ⚛️ Physics (Thread ID: 18)
  * 🌿 Environment (Thread ID: 19)
  * 📚 General Studies (Thread ID: 20)
  * 🛡️ Disaster Management (Thread ID: 21)
- Persisted all thread IDs into config.xlsx for quiz dispatching via send.js and schedule.js
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -399,12 +399,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F17"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,8 +434,8 @@
       <c r="B2" t="str">
         <v>📜</v>
       </c>
-      <c r="C2" t="str">
-        <v/>
+      <c r="C2">
+        <v>6</v>
       </c>
       <c r="D2" t="str">
         <v>0 9,18 * * *</v>
@@ -454,8 +454,8 @@
       <c r="B3" t="str">
         <v>🏛️</v>
       </c>
-      <c r="C3" t="str">
-        <v/>
+      <c r="C3">
+        <v>7</v>
       </c>
       <c r="D3" t="str">
         <v>0 */3 * * *</v>
@@ -474,8 +474,8 @@
       <c r="B4" t="str">
         <v>🌍</v>
       </c>
-      <c r="C4" t="str">
-        <v/>
+      <c r="C4">
+        <v>8</v>
       </c>
       <c r="D4" t="str">
         <v>0 */3 * * *</v>
@@ -494,8 +494,8 @@
       <c r="B5" t="str">
         <v>🗺️</v>
       </c>
-      <c r="C5" t="str">
-        <v/>
+      <c r="C5">
+        <v>9</v>
       </c>
       <c r="D5" t="str">
         <v>0 */3 * * *</v>
@@ -514,8 +514,8 @@
       <c r="B6" t="str">
         <v>💰</v>
       </c>
-      <c r="C6" t="str">
-        <v/>
+      <c r="C6">
+        <v>10</v>
       </c>
       <c r="D6" t="str">
         <v>0 */3 * * *</v>
@@ -534,8 +534,8 @@
       <c r="B7" t="str">
         <v>📈</v>
       </c>
-      <c r="C7" t="str">
-        <v/>
+      <c r="C7">
+        <v>11</v>
       </c>
       <c r="D7" t="str">
         <v>0 */3 * * *</v>
@@ -554,8 +554,8 @@
       <c r="B8" t="str">
         <v>⚖️</v>
       </c>
-      <c r="C8" t="str">
-        <v/>
+      <c r="C8">
+        <v>12</v>
       </c>
       <c r="D8" t="str">
         <v>0 */2 * * *</v>
@@ -574,8 +574,8 @@
       <c r="B9" t="str">
         <v>👥</v>
       </c>
-      <c r="C9" t="str">
-        <v/>
+      <c r="C9">
+        <v>13</v>
       </c>
       <c r="D9" t="str">
         <v>0 */4 * * *</v>
@@ -594,8 +594,8 @@
       <c r="B10" t="str">
         <v>📰</v>
       </c>
-      <c r="C10" t="str">
-        <v/>
+      <c r="C10">
+        <v>14</v>
       </c>
       <c r="D10" t="str">
         <v>0 8,14,20 * * *</v>
@@ -614,8 +614,8 @@
       <c r="B11" t="str">
         <v>🚀</v>
       </c>
-      <c r="C11" t="str">
-        <v/>
+      <c r="C11">
+        <v>15</v>
       </c>
       <c r="D11" t="str">
         <v>0 */3 * * *</v>
@@ -634,8 +634,8 @@
       <c r="B12" t="str">
         <v>🧬</v>
       </c>
-      <c r="C12" t="str">
-        <v/>
+      <c r="C12">
+        <v>16</v>
       </c>
       <c r="D12" t="str">
         <v>0 */4 * * *</v>
@@ -654,8 +654,8 @@
       <c r="B13" t="str">
         <v>🧪</v>
       </c>
-      <c r="C13" t="str">
-        <v/>
+      <c r="C13">
+        <v>17</v>
       </c>
       <c r="D13" t="str">
         <v>0 */4 * * *</v>
@@ -674,8 +674,8 @@
       <c r="B14" t="str">
         <v>⚛️</v>
       </c>
-      <c r="C14" t="str">
-        <v/>
+      <c r="C14">
+        <v>18</v>
       </c>
       <c r="D14" t="str">
         <v>0 */4 * * *</v>
@@ -694,8 +694,8 @@
       <c r="B15" t="str">
         <v>🌿</v>
       </c>
-      <c r="C15" t="str">
-        <v/>
+      <c r="C15">
+        <v>19</v>
       </c>
       <c r="D15" t="str">
         <v>0 */3 * * *</v>
@@ -714,8 +714,8 @@
       <c r="B16" t="str">
         <v>📚</v>
       </c>
-      <c r="C16" t="str">
-        <v/>
+      <c r="C16">
+        <v>20</v>
       </c>
       <c r="D16" t="str">
         <v>0 */3 * * *</v>
@@ -734,8 +734,8 @@
       <c r="B17" t="str">
         <v>🛡️</v>
       </c>
-      <c r="C17" t="str">
-        <v/>
+      <c r="C17">
+        <v>21</v>
       </c>
       <c r="D17" t="str">
         <v>0 */4 * * *</v>

</xml_diff>